<commit_message>
Simplify and fix the Excel automation
</commit_message>
<xml_diff>
--- a/src/examples/excel_automation.xlsx
+++ b/src/examples/excel_automation.xlsx
@@ -43,10 +43,10 @@
     <t xml:space="preserve">fc72b069-f3ee-36f5-9262-5d5310ae439a</t>
   </si>
   <si>
-    <t xml:space="preserve">rare earth oxides production, from rare earth carbonate concentrate | europium oxide | EN15804GD, U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">df779cb6-b80f-409a-805f-0f3c931f0ff4</t>
+    <t xml:space="preserve">rare earth oxides production, from rare earth carbonate concentrate | europium oxide | APOS, U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e2db2b12-19ed-30ef-a47c-941f84eb53e1</t>
   </si>
 </sst>
 </file>

</xml_diff>